<commit_message>
give the manifests a caller and fix the documented run order
</commit_message>
<xml_diff>
--- a/04_Figures/F06_prediction/c_data/results.xlsx
+++ b/04_Figures/F06_prediction/c_data/results.xlsx
@@ -59193,43 +59193,43 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" t="n">
         <v>14</v>
       </c>
       <c r="F3" t="n">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="G3" t="n">
         <v>200</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.144153434865446</v>
+        <v>0.620937211013559</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.797802197802198</v>
+        <v>0.87004616344005</v>
       </c>
       <c r="J3" t="n">
         <v>0.00497512437810945</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0099502487562189</v>
+        <v>0.00497512437810945</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.159951406304208</v>
+        <v>-1.01739479271618</v>
       </c>
       <c r="M3" t="n">
-        <v>0.00167682399869619</v>
+        <v>0.958346038400894</v>
       </c>
     </row>
     <row r="4">
@@ -59237,16 +59237,16 @@
         <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4" t="n">
         <v>79</v>
@@ -59255,10 +59255,10 @@
         <v>200</v>
       </c>
       <c r="H4" t="n">
-        <v>0.620937211013559</v>
+        <v>0.0331657929976628</v>
       </c>
       <c r="I4" t="n">
-        <v>0.87004616344005</v>
+        <v>0.25</v>
       </c>
       <c r="J4" t="n">
         <v>0.00497512437810945</v>
@@ -59267,10 +59267,10 @@
         <v>0.00497512437810945</v>
       </c>
       <c r="L4" t="n">
-        <v>-1.01739479271618</v>
+        <v>-0.148625885579399</v>
       </c>
       <c r="M4" t="n">
-        <v>0.958346038400894</v>
+        <v>0.0171809028068345</v>
       </c>
     </row>
     <row r="5">
@@ -59278,7 +59278,7 @@
         <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
         <v>27</v>
@@ -59287,36 +59287,36 @@
         <v>20</v>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" t="n">
-        <v>79</v>
+        <v>237</v>
       </c>
       <c r="G5" t="n">
         <v>200</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0331657929976628</v>
+        <v>0.077556765871716</v>
       </c>
       <c r="I5" t="n">
-        <v>0.25</v>
+        <v>0.415384615384615</v>
       </c>
       <c r="J5" t="n">
-        <v>0.00497512437810945</v>
+        <v>0.0099502487562189</v>
       </c>
       <c r="K5" t="n">
-        <v>0.00497512437810945</v>
+        <v>0.0099502487562189</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.148625885579399</v>
+        <v>-0.157106296210139</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0171809028068345</v>
+        <v>0.0457359998087378</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
         <v>33</v>
@@ -59325,22 +59325,22 @@
         <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E6" t="n">
         <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>237</v>
+        <v>5711</v>
       </c>
       <c r="G6" t="n">
         <v>200</v>
       </c>
       <c r="H6" t="n">
-        <v>0.077556765871716</v>
+        <v>0.0827563970827074</v>
       </c>
       <c r="I6" t="n">
-        <v>0.415384615384615</v>
+        <v>0.367032967032967</v>
       </c>
       <c r="J6" t="n">
         <v>0.0099502487562189</v>
@@ -59349,10 +59349,10 @@
         <v>0.0099502487562189</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.157106296210139</v>
+        <v>-0.175165333233226</v>
       </c>
       <c r="M6" t="n">
-        <v>0.0457359998087378</v>
+        <v>0.0904612030912077</v>
       </c>
     </row>
     <row r="7">
@@ -59366,7 +59366,7 @@
         <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E7" t="n">
         <v>14</v>
@@ -59378,104 +59378,104 @@
         <v>200</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0827563970827074</v>
+        <v>0.346859073593345</v>
       </c>
       <c r="I7" t="n">
-        <v>0.367032967032967</v>
+        <v>0.648351648351648</v>
       </c>
       <c r="J7" t="n">
         <v>0.0099502487562189</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0099502487562189</v>
+        <v>0.0149253731343284</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.175165333233226</v>
+        <v>-0.268049980556694</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0904612030912077</v>
+        <v>0.268834820382985</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C8" t="s">
         <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F8" t="n">
-        <v>5711</v>
+        <v>11</v>
       </c>
       <c r="G8" t="n">
         <v>200</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.0246271271692966</v>
+        <v>0.249732775292857</v>
       </c>
       <c r="I8" t="n">
-        <v>-0.107692307692308</v>
+        <v>0.457142857142857</v>
       </c>
       <c r="J8" t="n">
-        <v>0.0099502487562189</v>
+        <v>0.0149253731343284</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0149253731343284</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.161006234765979</v>
+        <v>-0.944401055961812</v>
       </c>
       <c r="M8" t="n">
-        <v>0.0183186735988543</v>
+        <v>2.9143487690887</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C9" t="s">
         <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F9" t="n">
-        <v>5711</v>
+        <v>11</v>
       </c>
       <c r="G9" t="n">
         <v>200</v>
       </c>
       <c r="H9" t="n">
-        <v>0.346859073593345</v>
+        <v>0.309257343662561</v>
       </c>
       <c r="I9" t="n">
-        <v>0.648351648351648</v>
+        <v>0.492857142857143</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0099502487562189</v>
+        <v>0.0149253731343284</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0149253731343284</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.268049980556694</v>
+        <v>-0.2675667632731</v>
       </c>
       <c r="M9" t="n">
-        <v>0.268834820382985</v>
+        <v>0.255420078321811</v>
       </c>
     </row>
     <row r="10">
@@ -59483,81 +59483,81 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C10" t="s">
         <v>27</v>
       </c>
       <c r="D10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F10" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G10" t="n">
         <v>200</v>
       </c>
       <c r="H10" t="n">
-        <v>0.249732775292857</v>
+        <v>0.282583392968293</v>
       </c>
       <c r="I10" t="n">
-        <v>0.457142857142857</v>
+        <v>0.463736263736264</v>
       </c>
       <c r="J10" t="n">
         <v>0.0149253731343284</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0149253731343284</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.944401055961812</v>
+        <v>-0.231537184185335</v>
       </c>
       <c r="M10" t="n">
-        <v>2.9143487690887</v>
+        <v>0.215716391897721</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
         <v>27</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E11" t="n">
         <v>15</v>
       </c>
       <c r="F11" t="n">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="G11" t="n">
         <v>200</v>
       </c>
       <c r="H11" t="n">
-        <v>0.309257343662561</v>
+        <v>0.407014128958588</v>
       </c>
       <c r="I11" t="n">
-        <v>0.492857142857143</v>
+        <v>0.603571428571428</v>
       </c>
       <c r="J11" t="n">
         <v>0.0149253731343284</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0447761194029851</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.2675667632731</v>
+        <v>-0.736577337708326</v>
       </c>
       <c r="M11" t="n">
-        <v>0.255420078321811</v>
+        <v>0.654777899967561</v>
       </c>
     </row>
     <row r="12">
@@ -59565,7 +59565,7 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
         <v>27</v>
@@ -59574,72 +59574,72 @@
         <v>16</v>
       </c>
       <c r="E12" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G12" t="n">
         <v>200</v>
       </c>
       <c r="H12" t="n">
-        <v>0.282583392968293</v>
+        <v>0.2160515511346</v>
       </c>
       <c r="I12" t="n">
-        <v>0.463736263736264</v>
+        <v>0.296428571428571</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0149253731343284</v>
+        <v>0.0199004975124378</v>
       </c>
       <c r="K12" t="n">
-        <v>0.0149253731343284</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.231537184185335</v>
+        <v>-0.976827376630532</v>
       </c>
       <c r="M12" t="n">
-        <v>0.215716391897721</v>
+        <v>2.9426978925868</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
         <v>27</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E13" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F13" t="n">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="G13" t="n">
         <v>200</v>
       </c>
       <c r="H13" t="n">
-        <v>0.407014128958588</v>
+        <v>0.262322625063435</v>
       </c>
       <c r="I13" t="n">
-        <v>0.603571428571428</v>
+        <v>0.520879120879121</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0149253731343284</v>
+        <v>0.0199004975124378</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.736577337708326</v>
+        <v>-0.263104470939312</v>
       </c>
       <c r="M13" t="n">
-        <v>0.654777899967561</v>
+        <v>0.325367879391364</v>
       </c>
     </row>
     <row r="14">
@@ -59647,45 +59647,45 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C14" t="s">
         <v>27</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E14" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G14" t="n">
         <v>200</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2160515511346</v>
+        <v>0.36795135249738</v>
       </c>
       <c r="I14" t="n">
-        <v>0.296428571428571</v>
+        <v>0.556043956043956</v>
       </c>
       <c r="J14" t="n">
         <v>0.0199004975124378</v>
       </c>
       <c r="K14" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0497512437810945</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.976827376630532</v>
+        <v>-0.655480593135721</v>
       </c>
       <c r="M14" t="n">
-        <v>2.9426978925868</v>
+        <v>0.709398093986986</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
         <v>33</v>
@@ -59694,116 +59694,116 @@
         <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E15" t="n">
         <v>14</v>
       </c>
       <c r="F15" t="n">
-        <v>33</v>
+        <v>237</v>
       </c>
       <c r="G15" t="n">
         <v>200</v>
       </c>
       <c r="H15" t="n">
-        <v>0.262322625063435</v>
+        <v>0.162702655113724</v>
       </c>
       <c r="I15" t="n">
-        <v>0.520879120879121</v>
+        <v>0.556043956043956</v>
       </c>
       <c r="J15" t="n">
         <v>0.0199004975124378</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0199004975124378</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.263104470939312</v>
+        <v>-0.192847165091876</v>
       </c>
       <c r="M15" t="n">
-        <v>0.325367879391364</v>
+        <v>0.136850848173076</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
         <v>27</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>33</v>
+        <v>1905</v>
       </c>
       <c r="G16" t="n">
         <v>200</v>
       </c>
       <c r="H16" t="n">
-        <v>0.36795135249738</v>
+        <v>0.294544129797594</v>
       </c>
       <c r="I16" t="n">
-        <v>0.556043956043956</v>
+        <v>0.603571428571428</v>
       </c>
       <c r="J16" t="n">
         <v>0.0199004975124378</v>
       </c>
       <c r="K16" t="n">
-        <v>0.0497512437810945</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.655480593135721</v>
+        <v>-0.348534688009132</v>
       </c>
       <c r="M16" t="n">
-        <v>0.709398093986986</v>
+        <v>0.352570601959223</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>79</v>
+        <v>1904</v>
       </c>
       <c r="G17" t="n">
         <v>200</v>
       </c>
       <c r="H17" t="n">
-        <v>-0.134440347262801</v>
+        <v>0.0781794329927804</v>
       </c>
       <c r="I17" t="n">
-        <v>-0.53803781323382</v>
+        <v>0.25</v>
       </c>
       <c r="J17" t="n">
         <v>0.0199004975124378</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0199004975124378</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="L17" t="n">
-        <v>-0.161770570697133</v>
+        <v>-0.167969769694151</v>
       </c>
       <c r="M17" t="n">
-        <v>0.0144270183301137</v>
+        <v>0.106185132221508</v>
       </c>
     </row>
     <row r="18">
@@ -59811,7 +59811,7 @@
         <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
         <v>27</v>
@@ -59820,39 +59820,39 @@
         <v>19</v>
       </c>
       <c r="E18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F18" t="n">
-        <v>237</v>
+        <v>79</v>
       </c>
       <c r="G18" t="n">
         <v>200</v>
       </c>
       <c r="H18" t="n">
-        <v>0.162702655113724</v>
+        <v>0.141303370516273</v>
       </c>
       <c r="I18" t="n">
-        <v>0.556043956043956</v>
+        <v>0.307142857142857</v>
       </c>
       <c r="J18" t="n">
-        <v>0.0199004975124378</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0199004975124378</v>
+        <v>0.0696517412935323</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.192847165091876</v>
+        <v>-0.186128616954252</v>
       </c>
       <c r="M18" t="n">
-        <v>0.136850848173076</v>
+        <v>0.149980207681085</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
         <v>27</v>
@@ -59864,36 +59864,36 @@
         <v>15</v>
       </c>
       <c r="F19" t="n">
-        <v>1905</v>
+        <v>79</v>
       </c>
       <c r="G19" t="n">
         <v>200</v>
       </c>
       <c r="H19" t="n">
-        <v>0.294544129797594</v>
+        <v>0.313843533454069</v>
       </c>
       <c r="I19" t="n">
-        <v>0.603571428571428</v>
+        <v>0.642857142857143</v>
       </c>
       <c r="J19" t="n">
-        <v>0.0199004975124378</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0298507462686567</v>
       </c>
       <c r="L19" t="n">
-        <v>-0.348534688009132</v>
+        <v>-0.765940371261893</v>
       </c>
       <c r="M19" t="n">
-        <v>0.352570601959223</v>
+        <v>0.67025304409798</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s">
         <v>27</v>
@@ -59902,31 +59902,31 @@
         <v>19</v>
       </c>
       <c r="E20" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F20" t="n">
-        <v>1904</v>
+        <v>79</v>
       </c>
       <c r="G20" t="n">
         <v>200</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0781794329927804</v>
+        <v>0.15644926634986</v>
       </c>
       <c r="I20" t="n">
-        <v>0.25</v>
+        <v>0.446153846153846</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0199004975124378</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="K20" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0298507462686567</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.167969769694151</v>
+        <v>-0.210244315236887</v>
       </c>
       <c r="M20" t="n">
-        <v>0.106185132221508</v>
+        <v>0.158645537090822</v>
       </c>
     </row>
     <row r="21">
@@ -59934,45 +59934,45 @@
         <v>34</v>
       </c>
       <c r="B21" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C21" t="s">
         <v>27</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E21" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F21" t="n">
-        <v>79</v>
+        <v>237</v>
       </c>
       <c r="G21" t="n">
         <v>200</v>
       </c>
       <c r="H21" t="n">
-        <v>0.141303370516273</v>
+        <v>0.259726105892755</v>
       </c>
       <c r="I21" t="n">
-        <v>0.307142857142857</v>
+        <v>0.525274725274725</v>
       </c>
       <c r="J21" t="n">
         <v>0.0248756218905473</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0696517412935323</v>
+        <v>0.0298507462686567</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.186128616954252</v>
+        <v>-0.186438934688261</v>
       </c>
       <c r="M21" t="n">
-        <v>0.149980207681085</v>
+        <v>0.138191298603544</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -59987,28 +59987,28 @@
         <v>15</v>
       </c>
       <c r="F22" t="n">
-        <v>79</v>
+        <v>1904</v>
       </c>
       <c r="G22" t="n">
         <v>200</v>
       </c>
       <c r="H22" t="n">
-        <v>0.313843533454069</v>
+        <v>0.363192449508588</v>
       </c>
       <c r="I22" t="n">
-        <v>0.642857142857143</v>
+        <v>0.564285714285714</v>
       </c>
       <c r="J22" t="n">
         <v>0.0248756218905473</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0298507462686567</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="L22" t="n">
-        <v>-0.765940371261893</v>
+        <v>-0.354960035781348</v>
       </c>
       <c r="M22" t="n">
-        <v>0.67025304409798</v>
+        <v>0.326203360581713</v>
       </c>
     </row>
     <row r="23">
@@ -60016,16 +60016,16 @@
         <v>34</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
         <v>27</v>
       </c>
       <c r="D23" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E23" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F23" t="n">
         <v>79</v>
@@ -60034,22 +60034,22 @@
         <v>200</v>
       </c>
       <c r="H23" t="n">
-        <v>0.15644926634986</v>
+        <v>0.230355806102047</v>
       </c>
       <c r="I23" t="n">
-        <v>0.446153846153846</v>
+        <v>0.432142857142857</v>
       </c>
       <c r="J23" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0298507462686567</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0298507462686567</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="L23" t="n">
-        <v>-0.210244315236887</v>
+        <v>-0.221781376753241</v>
       </c>
       <c r="M23" t="n">
-        <v>0.158645537090822</v>
+        <v>0.188495746472281</v>
       </c>
     </row>
     <row r="24">
@@ -60063,7 +60063,7 @@
         <v>27</v>
       </c>
       <c r="D24" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E24" t="n">
         <v>14</v>
@@ -60075,63 +60075,63 @@
         <v>200</v>
       </c>
       <c r="H24" t="n">
-        <v>0.259726105892755</v>
+        <v>0.411266403925074</v>
       </c>
       <c r="I24" t="n">
-        <v>0.525274725274725</v>
+        <v>0.67032967032967</v>
       </c>
       <c r="J24" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0298507462686567</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0298507462686567</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="L24" t="n">
-        <v>-0.186438934688261</v>
+        <v>-0.746450270442581</v>
       </c>
       <c r="M24" t="n">
-        <v>0.138191298603544</v>
+        <v>0.731814620750024</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C25" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E25" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F25" t="n">
-        <v>1904</v>
+        <v>237</v>
       </c>
       <c r="G25" t="n">
         <v>200</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.055026737045009</v>
+        <v>0.17778999080829</v>
       </c>
       <c r="I25" t="n">
-        <v>-0.0678571428571429</v>
+        <v>0.446153846153846</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="K25" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="L25" t="n">
-        <v>-0.147669118865169</v>
+        <v>-0.212031969926516</v>
       </c>
       <c r="M25" t="n">
-        <v>0.0460628161942599</v>
+        <v>0.192339074737823</v>
       </c>
     </row>
     <row r="26">
@@ -60139,122 +60139,122 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E26" t="n">
         <v>15</v>
       </c>
       <c r="F26" t="n">
-        <v>1904</v>
+        <v>1905</v>
       </c>
       <c r="G26" t="n">
         <v>200</v>
       </c>
       <c r="H26" t="n">
-        <v>0.363192449508588</v>
+        <v>0.354968331880092</v>
       </c>
       <c r="I26" t="n">
-        <v>0.564285714285714</v>
+        <v>0.728571428571428</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="K26" t="n">
         <v>0.0248756218905473</v>
       </c>
       <c r="L26" t="n">
-        <v>-0.354960035781348</v>
+        <v>-0.661298023947358</v>
       </c>
       <c r="M26" t="n">
-        <v>0.326203360581713</v>
+        <v>0.63906698410649</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D27" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E27" t="n">
         <v>15</v>
       </c>
       <c r="F27" t="n">
-        <v>79</v>
+        <v>1903</v>
       </c>
       <c r="G27" t="n">
         <v>200</v>
       </c>
       <c r="H27" t="n">
-        <v>0.230355806102047</v>
+        <v>0.49137091378704</v>
       </c>
       <c r="I27" t="n">
-        <v>0.432142857142857</v>
+        <v>0.752693006869287</v>
       </c>
       <c r="J27" t="n">
-        <v>0.0298507462686567</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="K27" t="n">
-        <v>0.0447761194029851</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="L27" t="n">
-        <v>-0.221781376753241</v>
+        <v>-0.72881175563384</v>
       </c>
       <c r="M27" t="n">
-        <v>0.188495746472281</v>
+        <v>0.727690509108903</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D28" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E28" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F28" t="n">
-        <v>79</v>
+        <v>5711</v>
       </c>
       <c r="G28" t="n">
         <v>200</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.12474196551672</v>
+        <v>0.531421486712578</v>
       </c>
       <c r="I28" t="n">
-        <v>-0.746428571428571</v>
+        <v>0.739521556317317</v>
       </c>
       <c r="J28" t="n">
-        <v>0.0298507462686567</v>
+        <v>0.0348258706467662</v>
       </c>
       <c r="K28" t="n">
-        <v>0.0398009950248756</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="L28" t="n">
-        <v>-0.149407896236868</v>
+        <v>-0.790720804628055</v>
       </c>
       <c r="M28" t="n">
-        <v>0.0360035578123072</v>
+        <v>0.880155756661792</v>
       </c>
     </row>
     <row r="29">
@@ -60262,40 +60262,40 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C29" t="s">
         <v>27</v>
       </c>
       <c r="D29" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E29" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F29" t="n">
-        <v>237</v>
+        <v>79</v>
       </c>
       <c r="G29" t="n">
         <v>200</v>
       </c>
       <c r="H29" t="n">
-        <v>0.411266403925074</v>
+        <v>0.0753610263277481</v>
       </c>
       <c r="I29" t="n">
-        <v>0.67032967032967</v>
+        <v>0.196428571428571</v>
       </c>
       <c r="J29" t="n">
-        <v>0.0298507462686567</v>
+        <v>0.0398009950248756</v>
       </c>
       <c r="K29" t="n">
-        <v>0.0447761194029851</v>
+        <v>0.054726368159204</v>
       </c>
       <c r="L29" t="n">
-        <v>-0.746450270442581</v>
+        <v>-0.217453055895912</v>
       </c>
       <c r="M29" t="n">
-        <v>0.731814620750024</v>
+        <v>0.203855982299521</v>
       </c>
     </row>
     <row r="30">
@@ -60303,16 +60303,16 @@
         <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="C30" t="s">
         <v>27</v>
       </c>
       <c r="D30" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E30" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F30" t="n">
         <v>11</v>
@@ -60321,22 +60321,22 @@
         <v>200</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.925900255153497</v>
+        <v>0.214388914026353</v>
       </c>
       <c r="I30" t="n">
-        <v>0.45</v>
+        <v>0.415384615384615</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="K30" t="n">
-        <v>0.0945273631840796</v>
+        <v>0.0796019900497512</v>
       </c>
       <c r="L30" t="n">
-        <v>-18.1471235764055</v>
+        <v>-0.602448388394728</v>
       </c>
       <c r="M30" t="n">
-        <v>14.3504982340663</v>
+        <v>0.486495872812373</v>
       </c>
     </row>
     <row r="31">
@@ -60344,40 +60344,40 @@
         <v>34</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D31" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E31" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F31" t="n">
-        <v>237</v>
+        <v>79</v>
       </c>
       <c r="G31" t="n">
         <v>200</v>
       </c>
       <c r="H31" t="n">
-        <v>0.17778999080829</v>
+        <v>0.268352077801062</v>
       </c>
       <c r="I31" t="n">
-        <v>0.446153846153846</v>
+        <v>0.622591894121817</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="K31" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="L31" t="n">
-        <v>-0.212031969926516</v>
+        <v>-0.913200580299731</v>
       </c>
       <c r="M31" t="n">
-        <v>0.192339074737823</v>
+        <v>0.913330156669448</v>
       </c>
     </row>
     <row r="32">
@@ -60385,40 +60385,40 @@
         <v>35</v>
       </c>
       <c r="B32" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C32" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D32" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E32" t="n">
         <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>1905</v>
+        <v>1904</v>
       </c>
       <c r="G32" t="n">
         <v>200</v>
       </c>
       <c r="H32" t="n">
-        <v>0.354968331880092</v>
+        <v>0.0656768811329532</v>
       </c>
       <c r="I32" t="n">
-        <v>0.728571428571428</v>
+        <v>0.282142857142857</v>
       </c>
       <c r="J32" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="K32" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.054726368159204</v>
       </c>
       <c r="L32" t="n">
-        <v>-0.661298023947358</v>
+        <v>-0.165629445834063</v>
       </c>
       <c r="M32" t="n">
-        <v>0.63906698410649</v>
+        <v>0.126548952102067</v>
       </c>
     </row>
     <row r="33">
@@ -60426,531 +60426,39 @@
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C33" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D33" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E33" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F33" t="n">
-        <v>1903</v>
+        <v>1905</v>
       </c>
       <c r="G33" t="n">
         <v>200</v>
       </c>
       <c r="H33" t="n">
-        <v>0.49137091378704</v>
+        <v>0.216816581856955</v>
       </c>
       <c r="I33" t="n">
-        <v>0.752693006869287</v>
+        <v>0.485714285714286</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0348258706467662</v>
+        <v>0.0447761194029851</v>
       </c>
       <c r="K33" t="n">
-        <v>0.0248756218905473</v>
+        <v>0.0696517412935323</v>
       </c>
       <c r="L33" t="n">
-        <v>-0.72881175563384</v>
+        <v>-0.405335179319281</v>
       </c>
       <c r="M33" t="n">
-        <v>0.727690509108903</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" t="s">
-        <v>33</v>
-      </c>
-      <c r="C34" t="s">
-        <v>24</v>
-      </c>
-      <c r="D34" t="s">
-        <v>21</v>
-      </c>
-      <c r="E34" t="n">
-        <v>14</v>
-      </c>
-      <c r="F34" t="n">
-        <v>5711</v>
-      </c>
-      <c r="G34" t="n">
-        <v>200</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.531421486712578</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0.739521556317317</v>
-      </c>
-      <c r="J34" t="n">
-        <v>0.0348258706467662</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="L34" t="n">
-        <v>-0.790720804628055</v>
-      </c>
-      <c r="M34" t="n">
-        <v>0.880155756661792</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s">
-        <v>13</v>
-      </c>
-      <c r="B35" t="s">
-        <v>30</v>
-      </c>
-      <c r="C35" t="s">
-        <v>15</v>
-      </c>
-      <c r="D35" t="s">
-        <v>20</v>
-      </c>
-      <c r="E35" t="n">
-        <v>15</v>
-      </c>
-      <c r="F35" t="n">
-        <v>11</v>
-      </c>
-      <c r="G35" t="n">
-        <v>200</v>
-      </c>
-      <c r="H35" t="n">
-        <v>-0.112354637327623</v>
-      </c>
-      <c r="I35" t="n">
-        <v>-0.560714285714286</v>
-      </c>
-      <c r="J35" t="n">
-        <v>0.0398009950248756</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0.0497512437810945</v>
-      </c>
-      <c r="L35" t="n">
-        <v>-0.235007281133059</v>
-      </c>
-      <c r="M35" t="n">
-        <v>0.604799103620348</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s">
-        <v>13</v>
-      </c>
-      <c r="B36" t="s">
-        <v>31</v>
-      </c>
-      <c r="C36" t="s">
-        <v>27</v>
-      </c>
-      <c r="D36" t="s">
-        <v>20</v>
-      </c>
-      <c r="E36" t="n">
-        <v>14</v>
-      </c>
-      <c r="F36" t="n">
-        <v>11</v>
-      </c>
-      <c r="G36" t="n">
-        <v>200</v>
-      </c>
-      <c r="H36" t="n">
-        <v>-0.0908985192850358</v>
-      </c>
-      <c r="I36" t="n">
-        <v>-0.485714285714286</v>
-      </c>
-      <c r="J36" t="n">
-        <v>0.0398009950248756</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0.0597014925373134</v>
-      </c>
-      <c r="L36" t="n">
-        <v>-0.19111716569569</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0.113941631222515</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s">
-        <v>34</v>
-      </c>
-      <c r="B37" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" t="s">
-        <v>27</v>
-      </c>
-      <c r="D37" t="s">
-        <v>17</v>
-      </c>
-      <c r="E37" t="n">
-        <v>15</v>
-      </c>
-      <c r="F37" t="n">
-        <v>79</v>
-      </c>
-      <c r="G37" t="n">
-        <v>200</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.0753610263277481</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.196428571428571</v>
-      </c>
-      <c r="J37" t="n">
-        <v>0.0398009950248756</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0.054726368159204</v>
-      </c>
-      <c r="L37" t="n">
-        <v>-0.217453055895912</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0.203855982299521</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s">
-        <v>35</v>
-      </c>
-      <c r="B38" t="s">
-        <v>31</v>
-      </c>
-      <c r="C38" t="s">
-        <v>27</v>
-      </c>
-      <c r="D38" t="s">
-        <v>20</v>
-      </c>
-      <c r="E38" t="n">
-        <v>14</v>
-      </c>
-      <c r="F38" t="n">
-        <v>1905</v>
-      </c>
-      <c r="G38" t="n">
-        <v>200</v>
-      </c>
-      <c r="H38" t="n">
-        <v>-0.121996025531108</v>
-      </c>
-      <c r="I38" t="n">
-        <v>-0.718681318681319</v>
-      </c>
-      <c r="J38" t="n">
-        <v>0.0398009950248756</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0.0597014925373134</v>
-      </c>
-      <c r="L38" t="n">
-        <v>-0.162138100409769</v>
-      </c>
-      <c r="M38" t="n">
-        <v>0.0358803464309054</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" t="s">
-        <v>27</v>
-      </c>
-      <c r="D39" t="s">
-        <v>16</v>
-      </c>
-      <c r="E39" t="n">
-        <v>14</v>
-      </c>
-      <c r="F39" t="n">
-        <v>5711</v>
-      </c>
-      <c r="G39" t="n">
-        <v>200</v>
-      </c>
-      <c r="H39" t="n">
-        <v>-0.121247342241043</v>
-      </c>
-      <c r="I39" t="n">
-        <v>-0.301098901098901</v>
-      </c>
-      <c r="J39" t="n">
-        <v>0.0398009950248756</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0.0199004975124378</v>
-      </c>
-      <c r="L39" t="n">
-        <v>-0.160852131319298</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0.0231917594800975</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="s">
-        <v>13</v>
-      </c>
-      <c r="B40" t="s">
-        <v>31</v>
-      </c>
-      <c r="C40" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" t="s">
-        <v>21</v>
-      </c>
-      <c r="E40" t="n">
-        <v>14</v>
-      </c>
-      <c r="F40" t="n">
-        <v>11</v>
-      </c>
-      <c r="G40" t="n">
-        <v>200</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0.214388914026353</v>
-      </c>
-      <c r="I40" t="n">
-        <v>0.415384615384615</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="K40" t="n">
-        <v>0.0796019900497512</v>
-      </c>
-      <c r="L40" t="n">
-        <v>-0.602448388394728</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0.486495872812373</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="s">
-        <v>34</v>
-      </c>
-      <c r="B41" t="s">
-        <v>32</v>
-      </c>
-      <c r="C41" t="s">
-        <v>23</v>
-      </c>
-      <c r="D41" t="s">
-        <v>22</v>
-      </c>
-      <c r="E41" t="n">
-        <v>13</v>
-      </c>
-      <c r="F41" t="n">
-        <v>79</v>
-      </c>
-      <c r="G41" t="n">
-        <v>200</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0.268352077801062</v>
-      </c>
-      <c r="I41" t="n">
-        <v>0.622591894121817</v>
-      </c>
-      <c r="J41" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="K41" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="L41" t="n">
-        <v>-0.913200580299731</v>
-      </c>
-      <c r="M41" t="n">
-        <v>0.913330156669448</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="s">
-        <v>35</v>
-      </c>
-      <c r="B42" t="s">
-        <v>14</v>
-      </c>
-      <c r="C42" t="s">
-        <v>15</v>
-      </c>
-      <c r="D42" t="s">
-        <v>20</v>
-      </c>
-      <c r="E42" t="n">
-        <v>15</v>
-      </c>
-      <c r="F42" t="n">
-        <v>1905</v>
-      </c>
-      <c r="G42" t="n">
-        <v>200</v>
-      </c>
-      <c r="H42" t="n">
-        <v>-0.133608784082024</v>
-      </c>
-      <c r="I42" t="n">
-        <v>-0.996428571428571</v>
-      </c>
-      <c r="J42" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="K42" t="n">
-        <v>0.258706467661692</v>
-      </c>
-      <c r="L42" t="n">
-        <v>-0.152842197352296</v>
-      </c>
-      <c r="M42" t="n">
-        <v>0.039049317436372</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="s">
-        <v>35</v>
-      </c>
-      <c r="B43" t="s">
-        <v>29</v>
-      </c>
-      <c r="C43" t="s">
-        <v>24</v>
-      </c>
-      <c r="D43" t="s">
-        <v>20</v>
-      </c>
-      <c r="E43" t="n">
-        <v>15</v>
-      </c>
-      <c r="F43" t="n">
-        <v>1904</v>
-      </c>
-      <c r="G43" t="n">
-        <v>200</v>
-      </c>
-      <c r="H43" t="n">
-        <v>-0.144021825690348</v>
-      </c>
-      <c r="I43" t="n">
-        <v>-0.844851543925991</v>
-      </c>
-      <c r="J43" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="K43" t="n">
-        <v>0.0845771144278607</v>
-      </c>
-      <c r="L43" t="n">
-        <v>-0.15324725672511</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0.0534040022136463</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="s">
-        <v>35</v>
-      </c>
-      <c r="B44" t="s">
-        <v>30</v>
-      </c>
-      <c r="C44" t="s">
-        <v>27</v>
-      </c>
-      <c r="D44" t="s">
-        <v>19</v>
-      </c>
-      <c r="E44" t="n">
-        <v>15</v>
-      </c>
-      <c r="F44" t="n">
-        <v>1904</v>
-      </c>
-      <c r="G44" t="n">
-        <v>200</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0.0656768811329532</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0.282142857142857</v>
-      </c>
-      <c r="J44" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="K44" t="n">
-        <v>0.054726368159204</v>
-      </c>
-      <c r="L44" t="n">
-        <v>-0.165629445834063</v>
-      </c>
-      <c r="M44" t="n">
-        <v>0.126548952102067</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="s">
-        <v>35</v>
-      </c>
-      <c r="B45" t="s">
-        <v>31</v>
-      </c>
-      <c r="C45" t="s">
-        <v>27</v>
-      </c>
-      <c r="D45" t="s">
-        <v>22</v>
-      </c>
-      <c r="E45" t="n">
-        <v>14</v>
-      </c>
-      <c r="F45" t="n">
-        <v>1905</v>
-      </c>
-      <c r="G45" t="n">
-        <v>200</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0.216816581856955</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0.485714285714286</v>
-      </c>
-      <c r="J45" t="n">
-        <v>0.0447761194029851</v>
-      </c>
-      <c r="K45" t="n">
-        <v>0.0696517412935323</v>
-      </c>
-      <c r="L45" t="n">
-        <v>-0.405335179319281</v>
-      </c>
-      <c r="M45" t="n">
         <v>0.401321867493841</v>
       </c>
     </row>

</xml_diff>